<commit_message>
aggiunta V4 di cui fare excel e file .mat
</commit_message>
<xml_diff>
--- a/FOLDER/EXCEL.xlsx
+++ b/FOLDER/EXCEL.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lachiara\Desktop\Uni_Andrea\Magistrale\Secondo_Anno\Controllo_Avanzato\Pipe_Matlab\FOLDER\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lachiara\Documents\GitHub\ControlloAvanzato\FOLDER\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8B52F26-C19F-4269-80ED-54BAABAAC548}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4EE7026C-61A4-4318-ABBF-2C98290504D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -432,10 +432,10 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -727,26 +727,26 @@
       </c>
     </row>
     <row r="3" spans="1:18" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="8" t="s">
-        <v>1</v>
-      </c>
-      <c r="B3" s="8"/>
-      <c r="C3" s="8"/>
-      <c r="D3" s="8"/>
-      <c r="E3" s="8"/>
-      <c r="F3" s="8"/>
-      <c r="G3" s="8"/>
-      <c r="H3" s="8"/>
-      <c r="I3" s="8"/>
-      <c r="J3" s="8"/>
-      <c r="K3" s="8"/>
-      <c r="L3" s="8"/>
-      <c r="M3" s="8"/>
-      <c r="N3" s="8"/>
-      <c r="O3" s="8"/>
-      <c r="P3" s="8"/>
-      <c r="Q3" s="8"/>
-      <c r="R3" s="8"/>
+      <c r="A3" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="9"/>
+      <c r="C3" s="9"/>
+      <c r="D3" s="9"/>
+      <c r="E3" s="9"/>
+      <c r="F3" s="9"/>
+      <c r="G3" s="9"/>
+      <c r="H3" s="9"/>
+      <c r="I3" s="9"/>
+      <c r="J3" s="9"/>
+      <c r="K3" s="9"/>
+      <c r="L3" s="9"/>
+      <c r="M3" s="9"/>
+      <c r="N3" s="9"/>
+      <c r="O3" s="9"/>
+      <c r="P3" s="9"/>
+      <c r="Q3" s="9"/>
+      <c r="R3" s="9"/>
     </row>
     <row r="4" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A4" s="2"/>
@@ -2259,26 +2259,26 @@
       </c>
     </row>
     <row r="31" spans="1:18" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="9" t="s">
+      <c r="A31" s="8" t="s">
         <v>45</v>
       </c>
-      <c r="B31" s="9"/>
-      <c r="C31" s="9"/>
-      <c r="D31" s="9"/>
-      <c r="E31" s="9"/>
-      <c r="F31" s="9"/>
-      <c r="G31" s="9"/>
-      <c r="H31" s="9"/>
-      <c r="I31" s="9"/>
-      <c r="J31" s="9"/>
-      <c r="K31" s="9"/>
-      <c r="L31" s="9"/>
-      <c r="M31" s="9"/>
-      <c r="N31" s="9"/>
-      <c r="O31" s="9"/>
-      <c r="P31" s="9"/>
-      <c r="Q31" s="9"/>
-      <c r="R31" s="9"/>
+      <c r="B31" s="8"/>
+      <c r="C31" s="8"/>
+      <c r="D31" s="8"/>
+      <c r="E31" s="8"/>
+      <c r="F31" s="8"/>
+      <c r="G31" s="8"/>
+      <c r="H31" s="8"/>
+      <c r="I31" s="8"/>
+      <c r="J31" s="8"/>
+      <c r="K31" s="8"/>
+      <c r="L31" s="8"/>
+      <c r="M31" s="8"/>
+      <c r="N31" s="8"/>
+      <c r="O31" s="8"/>
+      <c r="P31" s="8"/>
+      <c r="Q31" s="8"/>
+      <c r="R31" s="8"/>
     </row>
     <row r="32" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A32" s="2"/>
@@ -2805,7 +2805,7 @@
         <v>0</v>
       </c>
       <c r="H41" s="5">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I41" s="5">
         <v>0</v>
@@ -3791,26 +3791,26 @@
       </c>
     </row>
     <row r="59" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A59" s="9" t="s">
+      <c r="A59" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="B59" s="9"/>
-      <c r="C59" s="9"/>
-      <c r="D59" s="9"/>
-      <c r="E59" s="9"/>
-      <c r="F59" s="9"/>
-      <c r="G59" s="9"/>
-      <c r="H59" s="9"/>
-      <c r="I59" s="9"/>
-      <c r="J59" s="9"/>
-      <c r="K59" s="9"/>
-      <c r="L59" s="9"/>
-      <c r="M59" s="9"/>
-      <c r="N59" s="9"/>
-      <c r="O59" s="9"/>
-      <c r="P59" s="9"/>
-      <c r="Q59" s="9"/>
-      <c r="R59" s="9"/>
+      <c r="B59" s="8"/>
+      <c r="C59" s="8"/>
+      <c r="D59" s="8"/>
+      <c r="E59" s="8"/>
+      <c r="F59" s="8"/>
+      <c r="G59" s="8"/>
+      <c r="H59" s="8"/>
+      <c r="I59" s="8"/>
+      <c r="J59" s="8"/>
+      <c r="K59" s="8"/>
+      <c r="L59" s="8"/>
+      <c r="M59" s="8"/>
+      <c r="N59" s="8"/>
+      <c r="O59" s="8"/>
+      <c r="P59" s="8"/>
+      <c r="Q59" s="8"/>
+      <c r="R59" s="8"/>
     </row>
     <row r="60" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A60" s="2"/>
@@ -4331,13 +4331,13 @@
         <v>0</v>
       </c>
       <c r="F69" s="5">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G69" s="5">
         <v>0</v>
       </c>
       <c r="H69" s="5">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="I69" s="5">
         <v>0</v>
@@ -5323,26 +5323,26 @@
       </c>
     </row>
     <row r="87" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A87" s="9" t="s">
+      <c r="A87" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="B87" s="9"/>
-      <c r="C87" s="9"/>
-      <c r="D87" s="9"/>
-      <c r="E87" s="9"/>
-      <c r="F87" s="9"/>
-      <c r="G87" s="9"/>
-      <c r="H87" s="9"/>
-      <c r="I87" s="9"/>
-      <c r="J87" s="9"/>
-      <c r="K87" s="9"/>
-      <c r="L87" s="9"/>
-      <c r="M87" s="9"/>
-      <c r="N87" s="9"/>
-      <c r="O87" s="9"/>
-      <c r="P87" s="9"/>
-      <c r="Q87" s="9"/>
-      <c r="R87" s="9"/>
+      <c r="B87" s="8"/>
+      <c r="C87" s="8"/>
+      <c r="D87" s="8"/>
+      <c r="E87" s="8"/>
+      <c r="F87" s="8"/>
+      <c r="G87" s="8"/>
+      <c r="H87" s="8"/>
+      <c r="I87" s="8"/>
+      <c r="J87" s="8"/>
+      <c r="K87" s="8"/>
+      <c r="L87" s="8"/>
+      <c r="M87" s="8"/>
+      <c r="N87" s="8"/>
+      <c r="O87" s="8"/>
+      <c r="P87" s="8"/>
+      <c r="Q87" s="8"/>
+      <c r="R87" s="8"/>
     </row>
     <row r="88" spans="1:18" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A88" s="2"/>
@@ -6855,35 +6855,35 @@
       </c>
     </row>
     <row r="115" spans="1:27" x14ac:dyDescent="0.3">
-      <c r="A115" s="9" t="s">
+      <c r="A115" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="B115" s="9"/>
-      <c r="C115" s="9"/>
-      <c r="D115" s="9"/>
-      <c r="E115" s="9"/>
-      <c r="F115" s="9"/>
-      <c r="G115" s="9"/>
-      <c r="H115" s="9"/>
-      <c r="I115" s="9"/>
-      <c r="J115" s="9"/>
-      <c r="K115" s="9"/>
-      <c r="L115" s="9"/>
-      <c r="M115" s="9"/>
-      <c r="N115" s="9"/>
-      <c r="O115" s="9"/>
-      <c r="P115" s="9"/>
-      <c r="Q115" s="9"/>
-      <c r="R115" s="9"/>
-      <c r="S115" s="9"/>
-      <c r="T115" s="9"/>
-      <c r="U115" s="9"/>
-      <c r="V115" s="9"/>
-      <c r="W115" s="9"/>
-      <c r="X115" s="9"/>
-      <c r="Y115" s="9"/>
-      <c r="Z115" s="9"/>
-      <c r="AA115" s="9"/>
+      <c r="B115" s="8"/>
+      <c r="C115" s="8"/>
+      <c r="D115" s="8"/>
+      <c r="E115" s="8"/>
+      <c r="F115" s="8"/>
+      <c r="G115" s="8"/>
+      <c r="H115" s="8"/>
+      <c r="I115" s="8"/>
+      <c r="J115" s="8"/>
+      <c r="K115" s="8"/>
+      <c r="L115" s="8"/>
+      <c r="M115" s="8"/>
+      <c r="N115" s="8"/>
+      <c r="O115" s="8"/>
+      <c r="P115" s="8"/>
+      <c r="Q115" s="8"/>
+      <c r="R115" s="8"/>
+      <c r="S115" s="8"/>
+      <c r="T115" s="8"/>
+      <c r="U115" s="8"/>
+      <c r="V115" s="8"/>
+      <c r="W115" s="8"/>
+      <c r="X115" s="8"/>
+      <c r="Y115" s="8"/>
+      <c r="Z115" s="8"/>
+      <c r="AA115" s="8"/>
     </row>
     <row r="116" spans="1:27" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A116" s="2"/>
@@ -6995,7 +6995,7 @@
         <v>1</v>
       </c>
       <c r="J117" s="5">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="K117" s="5">
         <v>0</v>
@@ -7078,7 +7078,7 @@
         <v>1</v>
       </c>
       <c r="J118" s="6">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="K118" s="6">
         <v>0</v>
@@ -7133,25 +7133,25 @@
       </c>
     </row>
     <row r="119" spans="1:27" x14ac:dyDescent="0.3">
-      <c r="A119" s="9" t="s">
+      <c r="A119" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="B119" s="9"/>
-      <c r="C119" s="9"/>
-      <c r="D119" s="9"/>
-      <c r="E119" s="9"/>
-      <c r="F119" s="9"/>
-      <c r="G119" s="9"/>
-      <c r="H119" s="9"/>
-      <c r="I119" s="9"/>
-      <c r="J119" s="9"/>
-      <c r="K119" s="9"/>
-      <c r="L119" s="9"/>
-      <c r="M119" s="9"/>
-      <c r="N119" s="9"/>
-      <c r="O119" s="9"/>
-      <c r="P119" s="9"/>
-      <c r="Q119" s="9"/>
+      <c r="B119" s="8"/>
+      <c r="C119" s="8"/>
+      <c r="D119" s="8"/>
+      <c r="E119" s="8"/>
+      <c r="F119" s="8"/>
+      <c r="G119" s="8"/>
+      <c r="H119" s="8"/>
+      <c r="I119" s="8"/>
+      <c r="J119" s="8"/>
+      <c r="K119" s="8"/>
+      <c r="L119" s="8"/>
+      <c r="M119" s="8"/>
+      <c r="N119" s="8"/>
+      <c r="O119" s="8"/>
+      <c r="P119" s="8"/>
+      <c r="Q119" s="8"/>
     </row>
     <row r="120" spans="1:27" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A120" s="3" t="s">
@@ -7613,55 +7613,55 @@
     </row>
     <row r="134" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A134">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B134">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C134">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D134">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E134">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F134">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G134">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H134">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I134">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J134">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K134">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L134">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M134">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N134">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O134">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P134">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q134">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="135" spans="1:17" x14ac:dyDescent="0.3">

</xml_diff>